<commit_message>
Update responsive defect reports and add README
</commit_message>
<xml_diff>
--- a/Test-Cases/Responsive-Compatibility-Test-Matrix.xlsx
+++ b/Test-Cases/Responsive-Compatibility-Test-Matrix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\somya\Downloads\Somya Folder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\somya\Downloads\Somya Folder\SauceDemo - manual Qa project\saucedemo-manual-qa\Test-Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80129555-FFCC-4629-B9ED-B33FA3E86124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F268A3D-4FE0-4E50-B934-0C4731BC5B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{58DD61E6-2955-4DC1-B708-8D26A08ED4CD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="76">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -74,9 +74,6 @@
     <t>Login form, inputs, and buttons fit within the viewport without unintended overlap or clipping.</t>
   </si>
   <si>
-    <t>Not Run</t>
-  </si>
-  <si>
     <t>RC-002</t>
   </si>
   <si>
@@ -174,13 +171,141 @@
   </si>
   <si>
     <t>Dynamic Catalog content can be viewed and scrolled without unintended viewport-related layout issues.</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Evidence/Responsive-Compatibility/RC-008-Desktop.png</t>
+  </si>
+  <si>
+    <t>BUG-003</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Evidence/Responsive-Compatibility/RC-007-Desktop.png;BUG-004 evidence is documented separately.</t>
+  </si>
+  <si>
+    <t>BUG-004</t>
+  </si>
+  <si>
+    <t>Desktop: RC-001-Desktop.png; 
+Tablet: RC-001-Tablet.png; 
+Mobile: RC-001-Mobile-Login-Layout.png</t>
+  </si>
+  <si>
+    <t>Desktop: Product cards, images, names, prices, and buttons were visible without clipping, overlap, or unintended horizontal scrolling.
+Tablet: Product catalog layout passed all checks.
+Mobile: Excessive vertical spacing between the product description and the price/Add to Cart button was observed. The user must scroll down to view the price and access the Add to Cart button.</t>
+  </si>
+  <si>
+    <t>Desktop: RC-003-Desktop.png
+Tablet: RC-003-Tablet.png
+Mobile: RC-003-Mobile-Product-Card-Spacing.png</t>
+  </si>
+  <si>
+    <t>Desktop: Product sorting dropdown worked correctly, and products were sorted in ascending price order when Price (low to high) was selected.
+Tablet: Product sorting and layout checks passed.
+Mobile: Product sorting and layout checks passed.</t>
+  </si>
+  <si>
+    <t>Desktop: RC-004-Desktop.png
+Tablet: RC-004-Tablet-Product-Sorting.png 
+Mobile: RC-004-Mobile-Product-Sorting.png</t>
+  </si>
+  <si>
+    <t>Desktop: Add to Cart changed to Remove, the cart badge incremented, and removing the product restored Add to Cart and cleared the badge.
+Tablet: Add to Cart / Remove workflow and cart badge updates worked correctly.
+Mobile: Add to Cart / Remove workflow and cart badge updates worked correctly.</t>
+  </si>
+  <si>
+    <t>Desktop: Cart product information and controls were visible and accessible, with no clipping, overlap, or unintended horizontal scrolling.
+Tablet: Cart product information and controls were accessible. No layout issues were observed.
+Mobile: Cart product information and controls were accessible. No layout issues were observed.</t>
+  </si>
+  <si>
+    <t>Desktop: Checkout fields and Continue button were visible and usable. Empty-field validation was readable and did not obstruct the form. However, whitespace-only required values were accepted, reproducing the existing functional validation defect.
+Tablet: Checkout information fields and Continue button were visible and usable. Empty-field validation was readable and did not obstruct the form.
+Mobile: Checkout information fields and Continue button were visible and usable. Empty-field validation was readable and did not obstruct the form.
+Functional note: Whitespace-only required values were accepted, reproducing existing defect BUG-004.</t>
+  </si>
+  <si>
+    <t>Desktop: Product details, quantity, price, subtotal, tax, and total were visible and readable. Finish and Cancel buttons were accessible. No unintended clipping, overlap, or horizontal scrolling was observed
+Tablet &amp; Mobile: Checkout overview displayed correctly. Order details, prices, totals, and controls were accessible. No layout issues reported.</t>
+  </si>
+  <si>
+    <t>Desktop: The order confirmation message was fully visible and readable. The Back Home button was visible and usable. No unintended clipping, overlap, or horizontal scrolling was observed.
+Tablet &amp; Mobile: Order completion page displayed correctly. Confirmation message and navigation controls were accessible. No layout issues reported.</t>
+  </si>
+  <si>
+    <t>Desktop: RC-009-Desktop.png
+Tablet: RC-009-Tablet-Order-Completion.png
+Mobile: RC-009-Mobile-Order-Completion.png</t>
+  </si>
+  <si>
+    <t>Desktop: The navigation menu opened correctly, its options were visible and readable, and it closed successfully using the close icon. No unintended clipping or horizontal scrolling was observed.
+Tablet &amp; Mobile: Navigation menu opened and closed correctly. Options were accessible. No layout issues reported.</t>
+  </si>
+  <si>
+    <t>Desktop: After Reset App State was selected, the cart badge cleared, but the product button remained Remove instead of reverting to Add to cart.
+Tablet &amp; Mobile: Reset App State cleared the cart badge and cart contents, but the product button remained Remove until the page was refreshed.
+Additional observation: When Reset App State was triggered while remaining on the cart page, the cart badge disappeared but the product remained visible in the cart.</t>
+  </si>
+  <si>
+    <t>Desktop: RC-011-Desktop.png
+Tablet: RC-011-Tablet-Cart-Item-Remains-After-Reset.png
+Mobile: RC-011-Mobile-Cart-Item-Remains-After-Reset.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUG-002,BUG-005 </t>
+  </si>
+  <si>
+    <t>BUG-006</t>
+  </si>
+  <si>
+    <t>Desktop: Username and password fields and the Login button were fully visible. No clipping, overlap, or unintended horizontal scrolling was observed.
+Tablet: Login form displayed correctly, with no clipping, overlap, or unintended horizontal scrolling.
+Mobile: The login form was visible, but the accepted-user information section extended below the initially visible viewport. Further scrolling verification is required to determine whether all information remains accessible.</t>
+  </si>
+  <si>
+    <t>Actual Result / Observations:
+Desktop: The invalid-credentials validation message was partially clipped at the upper boundary of the red error container and was not fully readable.
+Tablet: Both empty-fields and invalid-credentials validation messages were clearly visible and readable.
+Mobile: The empty-fields validation message was clearly visible. The invalid-credentials message was partially clipped and was not fully readable.</t>
+  </si>
+  <si>
+    <t>Desktop:RC-002-Desktop-Empty-Fields-Validation.png and RC-002-Desktop-Invalid-Credentials-Validation.png
+Tablet: RC-002-Tablet-Empty-Fields-Validation.png and RC-002-Tablet-Invalid-Credentials-Validation.png
+Mobile: RC-002-Mobile-Empty-Fields-Validation.png and RC-002-Mobile-Invalid-Credentials-Validation.png</t>
+  </si>
+  <si>
+    <t>Desktop, Tablet, and Mobile: In the Lazy Load section, product images were clipped and duplicate products appeared during scrolling. In the Spinner and Slider sections, product images were also clipped. The image-clipping issue was observed across all three tested viewports.</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>BUG-007</t>
+  </si>
+  <si>
+    <t>Pending investigation — Mobile</t>
+  </si>
+  <si>
+    <t>Desktop:RC-012-Desktop-Lazy-Load-Image-Clipping.png, RC-012-Desktop-Slider-Image-Clipping.png and RC-012-Desktop-Spinner-Image-Clipping.png
+Tablet: RC-012-Tablet-Lazy-Load-Image-Clipping.png, RC-012-Tablet-Spinner-Image-Clipping.png and RC-012-Tablet-Slider-Image-Clipping.png
+Mobile: RC-012-Mobile-Lazy-Load-Image-Clipping.png, RC-012-Mobile-Spinner-Image-Clipping.png and RC-012-Mobile-Slider-Image-Clipping.png</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,6 +318,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -215,10 +353,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -554,42 +695,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{141E394E-E306-4B00-BA02-D18B9C43A154}">
-  <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr defaultColWidth="19.5546875" defaultRowHeight="93.6" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="12.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17" style="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5546875" style="1"/>
+    <col min="4" max="4" width="11.21875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="12.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="41.5546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14" style="1" customWidth="1"/>
+    <col min="9" max="9" width="33.33203125" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="19.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -600,233 +750,344 @@
         <v>11</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="144" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="D12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="D13" s="1" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>12</v>
+        <v>49</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>